<commit_message>
Privacy: strip email/ID columns from survey xlsx; move internal planning docs out of participant repo
</commit_message>
<xml_diff>
--- a/course-materials/survey/ankieta-2026-07-10.xlsx
+++ b/course-materials/survey/ankieta-2026-07-10.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -468,624 +468,540 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Submission ID</t>
+          <t>Submitted at</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Respondent ID</t>
+          <t>Jak oceniasz swój poziom zaawansowania w AI?</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Submitted at</t>
+          <t>Główny obszar Twojej pracy</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Jak oceniasz swój poziom zaawansowania w AI?</t>
+          <t>Języki z jakimi najczęściej pracujesz</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Główny obszar Twojej pracy</t>
+          <t>Główny system operacyjny, na którym pracujesz</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Języki z jakimi najczęściej pracujesz</t>
+          <t>Główny IDE / edytor kodu, z którego najczęściej korzystasz</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Główny system operacyjny, na którym pracujesz</t>
+          <t>Główne narzędzia CI/CD, Repozytoria kodu, Task management itp.</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Główny IDE / edytor kodu, z którego najczęściej korzystasz</t>
+          <t>Czy któreś z tych narzędzi są on premises / self hosting?</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Główne narzędzia CI/CD, Repozytoria kodu, Task management itp.</t>
+          <t>Z której chmury najczęściej korzystasz w pracy?</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Czy któreś z tych narzędzi są on premises / self hosting?</t>
+          <t>Rodzaj projektów z jakimi najczęściej pracujesz</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Z której chmury najczęściej korzystasz w pracy?</t>
+          <t>Jaki procent Twojego kodu jest obecnie generowany przez agentów AI?</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Rodzaj projektów z jakimi najczęściej pracujesz</t>
+          <t>Z jakich narzędzi AI korzystasz?</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Jaki procent Twojego kodu jest obecnie generowany przez agentów AI?</t>
+          <t>Które z tych narzędzi chcesz lepiej poznać na szkoleniu?</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Z jakich narzędzi AI korzystasz?</t>
+          <t>Które narzędzia AI posiadasz w wersji płatnej? (subskrypcje)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Które z tych narzędzi chcesz lepiej poznać na szkoleniu?</t>
+          <t>Rodzaj licencji</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Które narzędzia AI posiadasz w wersji płatnej? (subskrypcje)</t>
+          <t>Rodzaj licencji (Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Rodzaj licencji</t>
+          <t>Rodzaj licencji (Licencje prywatne)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Rodzaj licencji (Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę)</t>
+          <t>W jakich zastosowaniach używasz AI?</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Rodzaj licencji (Licencje prywatne)</t>
+          <t>Czy Twoja firma korzysta z AI?</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>W jakich zastosowaniach używasz AI?</t>
+          <t>Co chcesz wynieść z tego szkolenia? Twoja motywacja.</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Czy Twoja firma korzysta z AI?</t>
+          <t>Czy masz konkretne problemy lub procesy, które chcesz usprawnić?</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Co chcesz wynieść z tego szkolenia? Twoja motywacja.</t>
+          <t>Jakie umiejętności lub narzędzia szczególnie Cię interesują?</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Czy masz konkretne problemy lub procesy, które chcesz usprawnić?</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Jakie umiejętności lub narzędzia szczególnie Cię interesują?</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
           <t>Twoje imię</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Adres e-mail</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BEQZEvA</t>
+          <t>2026-07-06 09:46:51</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>XxNAqXe</t>
+          <t>Początkujący</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-06 09:46:51</t>
+          <t>Inne</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Początkujący</t>
+          <t>SQL, Python</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Inne</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SQL, Python</t>
+          <t>PyCharm</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>GitHub</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PyCharm</t>
+          <t>pomidor.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>nie korzystam</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>pomidor.</t>
+          <t>Desktop Apps, Aplikacje SaaS, Dashboards</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>nie korzystam</t>
+          <t>100</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Desktop Apps, Aplikacje SaaS, Dashboards</t>
+          <t>ChatGPT App, Claude Code</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Jestem świeżynka - nie programuje. korzystam tylko z różnych llm w postaci pisania promptów. Chętnie poznam Claude Code, n8n i coś co w codzienności na początek warto się nauczyć.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>ChatGPT App, Claude Code</t>
+          <t>ChatGPT Plus / Teams / Ultra / Enterprise, Gemini AI Pro / Ultra, Claude Code Pro / Max / Business / Enterprise</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Jestem świeżynka - nie programuje. korzystam tylko z różnych llm w postaci pisania promptów. Chętnie poznam Claude Code, n8n i coś co w codzienności na początek warto się nauczyć.</t>
+          <t>Licencje prywatne, Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>ChatGPT Plus / Teams / Ultra / Enterprise, Gemini AI Pro / Ultra, Claude Code Pro / Max / Business / Enterprise</t>
+          <t>true</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Licencje prywatne, Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
+          <t>true</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Generowanie Testów, Design, UX, UI, prawo, umowy, analiza tekstu</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Nie, ale planujemy</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Generowanie Testów, Design, UX, UI, prawo, umowy, analiza tekstu</t>
+          <t>Chcę poznać możliwości claude. Na razie tylko piszę prompty, pracuję z tekstem, tworze aplikacje, quizy i inne. Chcę poznać coś więcej.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Nie, ale planujemy</t>
+          <t>Chcę ruszyć. zobaczyć jak pracują profesjonaliści, zobaczyć możliwości.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Chcę poznać możliwości claude. Na razie tylko piszę prompty, pracuję z tekstem, tworze aplikacje, quizy i inne. Chcę poznać coś więcej.</t>
+          <t>Co można wycisnąć z claude do codziennej pracy i życia.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Chcę ruszyć. zobaczyć jak pracują profesjonaliści, zobaczyć możliwości.</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Co można wycisnąć z claude do codziennej pracy i życia.</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
           <t>Piotr</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>majewpio@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X5MEoA4</t>
+          <t>2026-07-06 10:05:07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eqoO77k</t>
+          <t>Początkujący</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-06 10:05:07</t>
+          <t>Back-End, DevOps</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Początkujący</t>
+          <t>SQL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Back-End, DevOps</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>InteliJ IDEA</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>InteliJ IDEA</t>
+          <t>GitHub, Bitbucket, Jira, Confluence, Jenkins</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GitHub, Bitbucket, Jira, Confluence, Jenkins</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Dashboards, Internal tools</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Dashboards, Internal tools</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>10</t>
+          <t>GitHub Copilot</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>GitHub Copilot</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>GitHub Copilot Pro / Pro+</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>GitHub Copilot Pro / Pro+</t>
+          <t>true</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
+          <t>false</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Autocomplete, Research</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>Tak, regularnie</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Autocomplete, Research</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Tak, regularnie</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
           <t>Lepsze poznanie narzędzi AI do automatyzacji codziennych zadań i usprawnienie procesów wewnątrz projektu</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Jakub</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>kubasienko@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rDrd9oR</t>
+          <t>2026-07-10 10:02:22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NpEEgoQ</t>
+          <t>Średnio zaaw.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-10 10:02:22</t>
+          <t>Back-End, Full-Stack</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Średnio zaaw.</t>
+          <t>Python, C++, SQL, Bash/Shell</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Back-End, Full-Stack</t>
+          <t>Linux</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Python, C++, SQL, Bash/Shell</t>
+          <t>PyCharm</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Linux</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PyCharm</t>
+          <t>GitHub, Jira, Confluence, Bitbucket, Argo Workflows, Jenkins</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GitHub, Jira, Confluence, Bitbucket, Argo Workflows, Jenkins</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Aplikacje SaaS, Desktop Apps, Games / 3D, Internal tools</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>30</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Aplikacje SaaS, Desktop Apps, Games / 3D, Internal tools</t>
+          <t>Claude Code, Mistral Vibe</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t xml:space="preserve">Claude Code - ponieważ jest najbardziej popularny w moim otoczeniu. Vibe - ponieważ jest europejską alternatywą dla narzędzi typu Claude. Interesują mnie też rozwiązania oparte o modele lokalne, np. Llama. </t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Claude Code, Mistral Vibe</t>
+          <t>Żadne</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claude Code - ponieważ jest najbardziej popularny w moim otoczeniu. Vibe - ponieważ jest europejską alternatywą dla narzędzi typu Claude. Interesują mnie też rozwiązania oparte o modele lokalne, np. Llama. </t>
+          <t>Licencje prywatne</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Żadne</t>
+          <t>false</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Licencje prywatne</t>
+          <t>true</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>AI Agent, Generowanie kodu, Generowanie Testów, Dokumentacja kodu, Research</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Dopiero zaczynamy</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>AI Agent, Generowanie kodu, Generowanie Testów, Dokumentacja kodu, Research</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Dopiero zaczynamy</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
           <t xml:space="preserve">Wzmocnienie mojego warsztatu o narzędzia, które usprawniają pracę, szczególnie jej "nudne" części jak pisanie testów. Umiejętność pisania kodu przy pomocy agentów daje przewagę konkurencyjną na obecnym rynku tworzenia oprogranowania i przyciąga potencjalnych pracodawców lub klientów. </t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Mikołaj</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>mikolaj.feliks@holisticon.pl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GeBopGz</t>
+          <t>2026-07-10 13:59:09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>xXgoorJ</t>
+          <t>Średnio zaaw.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-10 13:59:09</t>
+          <t>Back-End</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Średnio zaaw.</t>
+          <t>Java, JavaScript / TypeScript, SQL, Bash/Shell</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Back-End</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, JavaScript / TypeScript, SQL, Bash/Shell</t>
+          <t>InteliJ IDEA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>InteliJ IDEA</t>
+          <t>GitHub, Bitbucket, Jira, Azure DevOps, Jenkins</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GitHub, Bitbucket, Jira, Azure DevOps, Jenkins</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Internal tools</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Internal tools</t>
+          <t>Microsoft Copilot</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>Claude Code</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Microsoft Copilot</t>
+          <t>Żadne</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Claude Code</t>
+          <t>Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Żadne</t>
+          <t>true</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Licencje biznesowe / enterprise opłacane przez firmę / pracodawcę</t>
+          <t>false</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Nauka</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>W ograniczonym zakresie</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Nauka</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>W ograniczonym zakresie</t>
+          <t>Zapoznanie się z narzędziem Claude Code, jako ogólny wstęp do pracy z agentami AI.</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Zapoznanie się z narzędziem Claude Code, jako ogólny wstęp do pracy z agentami AI.</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr">
-        <is>
           <t>Generowanie kodu</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Daniel</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>kdstanaszek@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>